<commit_message>
Histoire : Structure & Mix = 2e drill optionnel depuis la tuile CA
Clarifie la place du Structure & Mix : hors fil principal, c'est le 2e drill du
cockpit depuis la tuile CA (« d'où vient le CA / comment financé »), à jouer
selon l'audience. Le drill principal reste CAC → Diagnostic → construction 2027.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/DEMO_ACTE1.xlsx
+++ b/eduservices/tagetik/DEMO_ACTE1.xlsx
@@ -1406,7 +1406,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>On CREUSE le CAC</t>
+          <t>On CREUSE le CAC (drill principal)</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>clic marque → funnel campus ; puis → construction 2027</t>
+          <t>clic tuile CAC ; clic marque → funnel campus ; puis → construction 2027</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Pilotage complémentaire</t>
+          <t>2e drill (OPTIONNEL) — le contexte</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1443,12 +1443,12 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>« Attention : 3 marques sont 100 % financées par l'OPCO — dépendance à surveiller. »</t>
+          <t>« D'où vient le CA et comment il est financé : 2 marques = 70 % du CA, et 3 marques 100 % OPCO — dépendance à surveiller. »</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>rapport à part (pas dans le flux d'accueil)</t>
+          <t>clic tuile CA → Structure &amp; Mix (selon l'audience, hors fil principal)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cockpit : ajouter Dépenses, corriger légende CAC + marge pt, supprimer Données
- Ajout tuile Dépenses acquisition (+10% YoY, ochre) -> le mécanisme est
  maintenant VISIBLE sur la grille : dépenses +10% > volume +6% -> CAC +3,7%.
- Légende CAC corrigée (les dépenses montent plus vite que le volume, pas le CAC).
- Marge YoY : bug d'unité corrigé -> +0,6 pt (fraction ×100) au lieu de 0,01 pt.
- Feuille Données supprimée : le cockpit porte ses valeurs brutes (inputs) et
  calcule Marge (EBITDA/CA) et CAC (dépenses/inscrits) en interne. Classeur = 4
  feuilles : Histoire, Cockpit, Diagnostic CAC, Structure & Mix.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/DEMO_ACTE1.xlsx
+++ b/eduservices/tagetik/DEMO_ACTE1.xlsx
@@ -11,7 +11,6 @@
     <sheet name="Cockpit" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Diagnostic CAC" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Structure &amp; Mix" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Données" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,15 +20,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
-    <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00,,&quot; M€&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00,,&quot; M€&quot;"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="&quot;▲ &quot;0.0%"/>
     <numFmt numFmtId="168" formatCode="&quot;▲ &quot;0.0&quot; pt&quot;"/>
     <numFmt numFmtId="169" formatCode="#,##0&quot; €&quot;"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,23 +85,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000A5A48"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="007D8B98"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="000A5A48"/>
       <sz val="9"/>
     </font>
@@ -132,7 +114,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00152230"/>
+      <color rgb="000000FF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -149,26 +131,25 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00152230"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00B3641C"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00B3641C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
       <color rgb="00B3641C"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00152230"/>
-      <sz val="9"/>
+      <color rgb="00B3641C"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -181,12 +162,19 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00152230"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00152230"/>
       <sz val="15"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <color rgb="000A5A48"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -235,7 +223,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -259,92 +247,76 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="167" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -435,7 +407,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Dépenses d'acquisition (+21%) décrochent au-dessus de l'activité (+12%)</a:t>
+              <a:t>Dépenses d'acquisition (+21%) décrochent au-dessus de l'activité (+12%) — sur 2 ans</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -447,38 +419,6 @@
         <ser>
           <idx val="0"/>
           <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Cockpit'!A20</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$19:$D$19</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$20:$D$20</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
           <tx>
             <strRef>
               <f>'Cockpit'!A21</f>
@@ -499,12 +439,44 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Cockpit'!$B$19:$D$19</f>
+              <f>'Cockpit'!$B$20:$D$20</f>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Cockpit'!$B$21:$D$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Cockpit'!A22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$20:$D$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$22:$D$22</f>
             </numRef>
           </val>
         </ser>
@@ -1344,7 +1316,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
+    <row r="6" ht="56" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>0</t>
@@ -1371,7 +1343,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
+    <row r="7" ht="56" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
           <t>1</t>
@@ -1384,12 +1356,12 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>COCKPIT d'atterrissage 2026 : bandeau CA/EBITDA/Marge + 6 tuiles KPI (finance &amp; commercial) + 1 graphe de tension</t>
+          <t>COCKPIT d'atterrissage 2026 : bandeau CA/EBITDA/Marge + tuiles KPI (finance &amp; commercial, dont Dépenses) + 1 graphe de tension</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>« Voilà où on en est : on progresse partout… sauf un point, le coût d'acquisition se dégrade. C'est le départ du budget 2027. »</t>
+          <t>« On progresse partout… mais les dépenses d'acquisition montent plus vite que le volume : le CAC se dégrade. C'est le départ du budget 2027. »</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1398,7 +1370,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="56" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
           <t>2</t>
@@ -1425,7 +1397,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="54" customHeight="1">
+    <row r="9" ht="56" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>~</t>
@@ -1452,7 +1424,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
+    <row r="10" ht="56" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>→</t>
@@ -1497,10 +1469,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -1544,17 +1516,17 @@
     </row>
     <row r="5">
       <c r="A5" s="14">
-        <f>Données!B7</f>
+        <f>D9</f>
         <v/>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14">
-        <f>Données!C7</f>
+        <f>D10</f>
         <v/>
       </c>
       <c r="D5" s="13" t="n"/>
       <c r="E5" s="15">
-        <f>Données!C7/Données!B7</f>
+        <f>D10/D9</f>
         <v/>
       </c>
       <c r="F5" s="13" t="n"/>
@@ -1609,17 +1581,14 @@
           <t>Chiffre d'affaires (€)</t>
         </is>
       </c>
-      <c r="B9" s="19">
-        <f>Données!B5</f>
-        <v/>
-      </c>
-      <c r="C9" s="19">
-        <f>Données!B6</f>
-        <v/>
-      </c>
-      <c r="D9" s="19">
-        <f>Données!B7</f>
-        <v/>
+      <c r="B9" s="19" t="n">
+        <v>20064725</v>
+      </c>
+      <c r="C9" s="19" t="n">
+        <v>21268606</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>22544725</v>
       </c>
       <c r="E9" s="20">
         <f>D9/C9-1</f>
@@ -1637,17 +1606,14 @@
           <t>EBITDA (€)</t>
         </is>
       </c>
-      <c r="B10" s="19">
-        <f>Données!C5</f>
-        <v/>
-      </c>
-      <c r="C10" s="19">
-        <f>Données!C6</f>
-        <v/>
-      </c>
-      <c r="D10" s="19">
-        <f>Données!C7</f>
-        <v/>
+      <c r="B10" s="19" t="n">
+        <v>2648550</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>2977604</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>3291530</v>
       </c>
       <c r="E10" s="20">
         <f>D10/C10-1</f>
@@ -1666,19 +1632,19 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>Données!C5/Données!B5</f>
+        <f>B10/B9</f>
         <v/>
       </c>
       <c r="C11" s="22">
-        <f>Données!C6/Données!B6</f>
+        <f>C10/C9</f>
         <v/>
       </c>
       <c r="D11" s="22">
-        <f>Données!C7/Données!B7</f>
+        <f>D10/D9</f>
         <v/>
       </c>
       <c r="E11" s="23">
-        <f>D11-C11</f>
+        <f>(D11-C11)*100</f>
         <v/>
       </c>
       <c r="F11" s="21" t="inlineStr">
@@ -1705,17 +1671,14 @@
           <t>Leads</t>
         </is>
       </c>
-      <c r="B13" s="24">
-        <f>Données!D5</f>
-        <v/>
-      </c>
-      <c r="C13" s="24">
-        <f>Données!D6</f>
-        <v/>
-      </c>
-      <c r="D13" s="24">
-        <f>Données!D7</f>
-        <v/>
+      <c r="B13" s="24" t="n">
+        <v>15305</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>16226</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>17197</v>
       </c>
       <c r="E13" s="20">
         <f>D13/C13-1</f>
@@ -1733,17 +1696,14 @@
           <t>Inscrits</t>
         </is>
       </c>
-      <c r="B14" s="24">
-        <f>Données!E5</f>
-        <v/>
-      </c>
-      <c r="C14" s="24">
-        <f>Données!E6</f>
-        <v/>
-      </c>
-      <c r="D14" s="24">
-        <f>Données!E7</f>
-        <v/>
+      <c r="B14" s="24" t="n">
+        <v>1092</v>
+      </c>
+      <c r="C14" s="24" t="n">
+        <v>1159</v>
+      </c>
+      <c r="D14" s="24" t="n">
+        <v>1229</v>
       </c>
       <c r="E14" s="20">
         <f>D14/C14-1</f>
@@ -1758,103 +1718,128 @@
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
+          <t>Dépenses acquisition (€)</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>358819</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>394702</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>434174</v>
+      </c>
+      <c r="E15" s="26">
+        <f>D15/C15-1</f>
+        <v/>
+      </c>
+      <c r="F15" s="27" t="inlineStr">
+        <is>
+          <t>à surveiller</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
+        <is>
           <t>CAC (€/inscrit)</t>
         </is>
       </c>
-      <c r="B15" s="26">
-        <f>Données!F5/Données!E5</f>
-        <v/>
-      </c>
-      <c r="C15" s="26">
-        <f>Données!F6/Données!E6</f>
-        <v/>
-      </c>
-      <c r="D15" s="26">
-        <f>Données!F7/Données!E7</f>
-        <v/>
-      </c>
-      <c r="E15" s="27">
-        <f>D15/C15-1</f>
-        <v/>
-      </c>
-      <c r="F15" s="28" t="inlineStr">
+      <c r="B16" s="28">
+        <f>B15/B14</f>
+        <v/>
+      </c>
+      <c r="C16" s="28">
+        <f>C15/C14</f>
+        <v/>
+      </c>
+      <c r="D16" s="28">
+        <f>D15/D14</f>
+        <v/>
+      </c>
+      <c r="E16" s="26">
+        <f>D16/C16-1</f>
+        <v/>
+      </c>
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>à surveiller</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>CAC = seul KPI en tension : le coût d'acquisition monte plus vite que le volume. C'est ce que le budget 2027 doit corriger.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="29" t="inlineStr">
-        <is>
-          <t>TENSION — base 100 en 2024</t>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>CAC +3,7 % : les dépenses (+10 %) montent plus vite que le volume (+6 %) → chaque inscrit coûte un peu plus. Enjeu 2027 : croître SANS laisser filer le CAC.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
+          <t>TENSION — base 100 en 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
           <t>Année</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n">
+      <c r="B20" s="32" t="n">
         <v>2024</v>
       </c>
-      <c r="C19" s="31" t="n">
+      <c r="C20" s="32" t="n">
         <v>2025</v>
       </c>
-      <c r="D19" s="31" t="n">
+      <c r="D20" s="32" t="n">
         <v>2026</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="33" t="inlineStr">
         <is>
           <t>Activité (CA)</t>
         </is>
       </c>
-      <c r="B20" s="33">
-        <f>Données!B5/Données!B5*100</f>
-        <v/>
-      </c>
-      <c r="C20" s="33">
-        <f>Données!B6/Données!B5*100</f>
-        <v/>
-      </c>
-      <c r="D20" s="33">
-        <f>Données!B7/Données!B5*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="B21" s="34">
+        <f>B9/$B9*100</f>
+        <v/>
+      </c>
+      <c r="C21" s="34">
+        <f>C9/$B9*100</f>
+        <v/>
+      </c>
+      <c r="D21" s="34">
+        <f>D9/$B9*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Dépenses acq.</t>
         </is>
       </c>
-      <c r="B21" s="33">
-        <f>Données!F5/Données!F5*100</f>
-        <v/>
-      </c>
-      <c r="C21" s="33">
-        <f>Données!F6/Données!F5*100</f>
-        <v/>
-      </c>
-      <c r="D21" s="33">
-        <f>Données!F7/Données!F5*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="34" t="inlineStr">
-        <is>
-          <t>L'écart entre les 2 courbes = la dégradation du CAC → ce que le budget 2027 doit corriger. Clic tuile CAC → Diagnostic.</t>
+      <c r="B22" s="34">
+        <f>B15/$B15*100</f>
+        <v/>
+      </c>
+      <c r="C22" s="34">
+        <f>C15/$B15*100</f>
+        <v/>
+      </c>
+      <c r="D22" s="34">
+        <f>D15/$B15*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>Ici on VOIT le mécanisme : les dépenses montent plus vite que le CA. Clic tuile CAC → Diagnostic (funnel + CAC par marque).</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1909,7 @@
           <t>Leads</t>
         </is>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="24" t="n">
         <v>17197</v>
       </c>
     </row>
@@ -1934,10 +1919,10 @@
           <t>Candidatures</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="24" t="n">
         <v>3720</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="38">
         <f>B7/B6</f>
         <v/>
       </c>
@@ -1948,10 +1933,10 @@
           <t>Admis</t>
         </is>
       </c>
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="24" t="n">
         <v>2623</v>
       </c>
-      <c r="C8" s="39">
+      <c r="C8" s="38">
         <f>B8/B7</f>
         <v/>
       </c>
@@ -1962,21 +1947,21 @@
           <t>Inscrits</t>
         </is>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="24" t="n">
         <v>1229</v>
       </c>
-      <c r="C9" s="39">
+      <c r="C9" s="38">
         <f>B9/B8</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="40" t="inlineStr">
+      <c r="A10" s="39" t="inlineStr">
         <is>
           <t>Global lead → inscrit</t>
         </is>
       </c>
-      <c r="C10" s="41">
+      <c r="C10" s="40">
         <f>B9/B6</f>
         <v/>
       </c>
@@ -2016,13 +2001,13 @@
           <t>MBway</t>
         </is>
       </c>
-      <c r="B15" s="42" t="n">
+      <c r="B15" s="19" t="n">
         <v>166530</v>
       </c>
-      <c r="C15" s="38" t="n">
+      <c r="C15" s="24" t="n">
         <v>510</v>
       </c>
-      <c r="D15" s="43">
+      <c r="D15" s="41">
         <f>B15/C15</f>
         <v/>
       </c>
@@ -2033,13 +2018,13 @@
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="B16" s="42" t="n">
+      <c r="B16" s="19" t="n">
         <v>108103</v>
       </c>
-      <c r="C16" s="38" t="n">
+      <c r="C16" s="24" t="n">
         <v>338</v>
       </c>
-      <c r="D16" s="43">
+      <c r="D16" s="41">
         <f>B16/C16</f>
         <v/>
       </c>
@@ -2050,13 +2035,13 @@
           <t>IPAC</t>
         </is>
       </c>
-      <c r="B17" s="42" t="n">
+      <c r="B17" s="19" t="n">
         <v>51871</v>
       </c>
-      <c r="C17" s="38" t="n">
+      <c r="C17" s="24" t="n">
         <v>130</v>
       </c>
-      <c r="D17" s="43">
+      <c r="D17" s="41">
         <f>B17/C17</f>
         <v/>
       </c>
@@ -2067,13 +2052,13 @@
           <t>Pigier</t>
         </is>
       </c>
-      <c r="B18" s="42" t="n">
+      <c r="B18" s="19" t="n">
         <v>58580</v>
       </c>
-      <c r="C18" s="38" t="n">
+      <c r="C18" s="24" t="n">
         <v>164</v>
       </c>
-      <c r="D18" s="43">
+      <c r="D18" s="41">
         <f>B18/C18</f>
         <v/>
       </c>
@@ -2084,24 +2069,24 @@
           <t>Tunon</t>
         </is>
       </c>
-      <c r="B19" s="42" t="n">
+      <c r="B19" s="19" t="n">
         <v>49090</v>
       </c>
-      <c r="C19" s="38" t="n">
+      <c r="C19" s="24" t="n">
         <v>87</v>
       </c>
-      <c r="D19" s="44">
+      <c r="D19" s="42">
         <f>B19/C19</f>
         <v/>
       </c>
-      <c r="E19" s="45" t="inlineStr">
+      <c r="E19" s="43" t="inlineStr">
         <is>
           <t>◄ 1,7× la moyenne</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="34" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Le funnel dit COMMENT (taux) ; le CAC par marque dit OÙ agir → Tunon en priorité. Clic marque → funnel du campus.</t>
         </is>
@@ -2178,13 +2163,13 @@
           <t>MBway</t>
         </is>
       </c>
-      <c r="B6" s="42" t="n">
+      <c r="B6" s="19" t="n">
         <v>1995975</v>
       </c>
-      <c r="C6" s="42" t="n">
+      <c r="C6" s="19" t="n">
         <v>7525580</v>
       </c>
-      <c r="D6" s="46">
+      <c r="D6" s="44">
         <f>C6/(B6+C6)</f>
         <v/>
       </c>
@@ -2195,13 +2180,13 @@
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="B7" s="42" t="n">
+      <c r="B7" s="19" t="n">
         <v>1310700</v>
       </c>
-      <c r="C7" s="42" t="n">
+      <c r="C7" s="19" t="n">
         <v>4951430</v>
       </c>
-      <c r="D7" s="46">
+      <c r="D7" s="44">
         <f>C7/(B7+C7)</f>
         <v/>
       </c>
@@ -2212,17 +2197,17 @@
           <t>IPAC</t>
         </is>
       </c>
-      <c r="B8" s="42" t="n">
+      <c r="B8" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="42" t="n">
+      <c r="C8" s="19" t="n">
         <v>2571100</v>
       </c>
-      <c r="D8" s="41">
+      <c r="D8" s="40">
         <f>C8/(B8+C8)</f>
         <v/>
       </c>
-      <c r="E8" s="45" t="inlineStr">
+      <c r="E8" s="43" t="inlineStr">
         <is>
           <t>100 % OPCO</t>
         </is>
@@ -2234,17 +2219,17 @@
           <t>Pigier</t>
         </is>
       </c>
-      <c r="B9" s="42" t="n">
+      <c r="B9" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="42" t="n">
+      <c r="C9" s="19" t="n">
         <v>2137460</v>
       </c>
-      <c r="D9" s="41">
+      <c r="D9" s="40">
         <f>C9/(B9+C9)</f>
         <v/>
       </c>
-      <c r="E9" s="45" t="inlineStr">
+      <c r="E9" s="43" t="inlineStr">
         <is>
           <t>100 % OPCO</t>
         </is>
@@ -2256,17 +2241,17 @@
           <t>Tunon</t>
         </is>
       </c>
-      <c r="B10" s="42" t="n">
+      <c r="B10" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="42" t="n">
+      <c r="C10" s="19" t="n">
         <v>1941870</v>
       </c>
-      <c r="D10" s="41">
+      <c r="D10" s="40">
         <f>C10/(B10+C10)</f>
         <v/>
       </c>
-      <c r="E10" s="45" t="inlineStr">
+      <c r="E10" s="43" t="inlineStr">
         <is>
           <t>100 % OPCO</t>
         </is>
@@ -2297,7 +2282,7 @@
           <t>MBway</t>
         </is>
       </c>
-      <c r="B15" s="42" t="n">
+      <c r="B15" s="19" t="n">
         <v>9567455</v>
       </c>
     </row>
@@ -2307,7 +2292,7 @@
           <t>ISCOM</t>
         </is>
       </c>
-      <c r="B16" s="42" t="n">
+      <c r="B16" s="19" t="n">
         <v>6292550</v>
       </c>
     </row>
@@ -2317,7 +2302,7 @@
           <t>IPAC</t>
         </is>
       </c>
-      <c r="B17" s="42" t="n">
+      <c r="B17" s="19" t="n">
         <v>2582800</v>
       </c>
     </row>
@@ -2327,7 +2312,7 @@
           <t>Pigier</t>
         </is>
       </c>
-      <c r="B18" s="42" t="n">
+      <c r="B18" s="19" t="n">
         <v>2152220</v>
       </c>
     </row>
@@ -2337,12 +2322,12 @@
           <t>Tunon</t>
         </is>
       </c>
-      <c r="B19" s="42" t="n">
+      <c r="B19" s="19" t="n">
         <v>1949700</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="34" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>INSIGHT DAF : groupe massivement financé par l'alternance (OPCO). MBway/ISCOM ~79%, les 3 autres 100%. Dépendance à surveiller.</t>
         </is>
@@ -2352,138 +2337,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="36" t="inlineStr">
-        <is>
-          <t>DONNÉES — agrégats annuels groupe (compta produits + socle CRM)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="47" t="inlineStr">
-        <is>
-          <t>2024-2025 réalisé · 2026 atterrissage. Bleu = donnée.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Exercice</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Leads</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Inscrits</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Dépense acq.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="48" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B5" s="49" t="n">
-        <v>20064725</v>
-      </c>
-      <c r="C5" s="49" t="n">
-        <v>2648550</v>
-      </c>
-      <c r="D5" s="50" t="n">
-        <v>15305</v>
-      </c>
-      <c r="E5" s="50" t="n">
-        <v>1092</v>
-      </c>
-      <c r="F5" s="49" t="n">
-        <v>358819</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="48" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="B6" s="49" t="n">
-        <v>21268606</v>
-      </c>
-      <c r="C6" s="49" t="n">
-        <v>2977604</v>
-      </c>
-      <c r="D6" s="50" t="n">
-        <v>16226</v>
-      </c>
-      <c r="E6" s="50" t="n">
-        <v>1159</v>
-      </c>
-      <c r="F6" s="49" t="n">
-        <v>394702</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="48" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="B7" s="49" t="n">
-        <v>22544725</v>
-      </c>
-      <c r="C7" s="49" t="n">
-        <v>3291530</v>
-      </c>
-      <c r="D7" s="50" t="n">
-        <v>17197</v>
-      </c>
-      <c r="E7" s="50" t="n">
-        <v>1229</v>
-      </c>
-      <c r="F7" s="49" t="n">
-        <v>434174</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Meilleurs graphes : combo inscrits/CAC (cockpit) + bridge du CAC (diagnostic)
- Cockpit : le graphe base 100 (abstrait) remplacé par un COMBO valeurs réelles —
  barres = inscrits (volume), courbe = CAC (€, 2e axe). On voit le volume monter
  ET le coût unitaire grimper.
- Diagnostic : ajout du BRIDGE du CAC (waterfall) qui décompose la hausse 341->353
  en +34 € effet dépenses et -21 € effet volume (net +13 €). Formules -> réconcilie
  exactement. C'est la preuve visuelle que l'effet dépenses > l'effet volume.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/DEMO_ACTE1.xlsx
+++ b/eduservices/tagetik/DEMO_ACTE1.xlsx
@@ -19,16 +19,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0.00,,&quot; M€&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="&quot;▲ &quot;0.0%"/>
     <numFmt numFmtId="168" formatCode="&quot;▲ &quot;0.0&quot; pt&quot;"/>
     <numFmt numFmtId="169" formatCode="#,##0&quot; €&quot;"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -181,6 +180,21 @@
       <b val="1"/>
       <color rgb="00B3641C"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="007D8B98"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="5">
@@ -223,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -291,12 +305,12 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -316,6 +330,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="27" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -407,15 +430,16 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Dépenses d'acquisition (+21%) décrochent au-dessus de l'activité (+12%) — sur 2 ans</a:t>
+              <a:t>Volume (inscrits, barres) vs coût par inscrit (CAC, courbe)</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -425,7 +449,43 @@
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill>
+              <a:srgbClr val="E4F0EC"/>
+            </a:solidFill>
             <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$20:$D$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$21:$D$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Cockpit'!A22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="28000">
+              <a:solidFill>
+                <a:srgbClr val="B3641C"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -437,43 +497,6 @@
               </a:ln>
             </spPr>
           </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$20:$D$20</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$21:$D$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Cockpit'!A22</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$20:$D$20</f>
-            </numRef>
-          </cat>
           <val>
             <numRef>
               <f>'Cockpit'!$B$22:$D$22</f>
@@ -481,7 +504,7 @@
           </val>
         </ser>
         <axId val="10"/>
-        <axId val="100"/>
+        <axId val="200"/>
       </lineChart>
       <catAx>
         <axId val="10"/>
@@ -501,9 +524,51 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Inscrits</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>CAC (€)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
@@ -675,6 +740,147 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
+              <a:t>Bridge du CAC : +34 € (dépenses) − 21 € (volume) = +13 € net</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="FFFFFF"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Diagnostic CAC'!$A$30:$A$33</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Diagnostic CAC'!$B$30:$B$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="9AA7B0"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="B3641C"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="0D7A62"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="3"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="3D4F8F"/>
+              </a:solidFill>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <cat>
+            <numRef>
+              <f>'Diagnostic CAC'!$A$30:$A$33</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Diagnostic CAC'!$C$30:$C$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
               <a:t>Mix initiale / alternance : 3 marques 100% OPCO</a:t>
             </a:r>
           </a:p>
@@ -770,7 +976,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -912,6 +1118,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1778,68 +2006,63 @@
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>TENSION — base 100 en 2024</t>
+          <t>TENSION — le volume monte, mais le coût unitaire aussi</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="31" t="inlineStr">
-        <is>
-          <t>Année</t>
-        </is>
-      </c>
-      <c r="B20" s="32" t="n">
+      <c r="B20" s="31" t="n">
         <v>2024</v>
       </c>
-      <c r="C20" s="32" t="n">
+      <c r="C20" s="31" t="n">
         <v>2025</v>
       </c>
-      <c r="D20" s="32" t="n">
+      <c r="D20" s="31" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>Activité (CA)</t>
-        </is>
-      </c>
-      <c r="B21" s="34">
-        <f>B9/$B9*100</f>
-        <v/>
-      </c>
-      <c r="C21" s="34">
-        <f>C9/$B9*100</f>
-        <v/>
-      </c>
-      <c r="D21" s="34">
-        <f>D9/$B9*100</f>
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>Inscrits</t>
+        </is>
+      </c>
+      <c r="B21" s="33">
+        <f>B14</f>
+        <v/>
+      </c>
+      <c r="C21" s="33">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="D21" s="33">
+        <f>D14</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>Dépenses acq.</t>
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>CAC (€)</t>
         </is>
       </c>
       <c r="B22" s="34">
-        <f>B15/$B15*100</f>
+        <f>B16</f>
         <v/>
       </c>
       <c r="C22" s="34">
-        <f>C15/$B15*100</f>
+        <f>C16</f>
         <v/>
       </c>
       <c r="D22" s="34">
-        <f>D15/$B15*100</f>
+        <f>D16</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>Ici on VOIT le mécanisme : les dépenses montent plus vite que le CA. Clic tuile CAC → Diagnostic (funnel + CAC par marque).</t>
+          <t>Les inscrits progressent (barres) mais le CAC grimpe (courbe) : les dépenses montent plus vite que le volume. Clic tuile CAC → Diagnostic.</t>
         </is>
       </c>
     </row>
@@ -1855,14 +2078,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2089,6 +2313,110 @@
       <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Le funnel dit COMMENT (taux) ; le CAC par marque dit OÙ agir → Tunon en priorité. Clic marque → funnel du campus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="36" t="inlineStr">
+        <is>
+          <t>Bridge du CAC — d'où vient la hausse 2025 → 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="44" t="inlineStr">
+        <is>
+          <t>CAC 2025</t>
+        </is>
+      </c>
+      <c r="B30" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="46">
+        <f>F30/F32</f>
+        <v/>
+      </c>
+      <c r="E30" s="47" t="inlineStr">
+        <is>
+          <t>Dépenses 2025</t>
+        </is>
+      </c>
+      <c r="F30" s="48" t="n">
+        <v>394702</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="44" t="inlineStr">
+        <is>
+          <t>+ Effet dépenses</t>
+        </is>
+      </c>
+      <c r="B31" s="45">
+        <f>F30/F32</f>
+        <v/>
+      </c>
+      <c r="C31" s="46">
+        <f>(F31-F30)/F32</f>
+        <v/>
+      </c>
+      <c r="E31" s="47" t="inlineStr">
+        <is>
+          <t>Dépenses 2026</t>
+        </is>
+      </c>
+      <c r="F31" s="48" t="n">
+        <v>434174</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="44" t="inlineStr">
+        <is>
+          <t>− Effet volume</t>
+        </is>
+      </c>
+      <c r="B32" s="45">
+        <f>F31/F33</f>
+        <v/>
+      </c>
+      <c r="C32" s="46">
+        <f>F31/F32-F31/F33</f>
+        <v/>
+      </c>
+      <c r="E32" s="47" t="inlineStr">
+        <is>
+          <t>Inscrits 2025</t>
+        </is>
+      </c>
+      <c r="F32" s="48" t="n">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="44" t="inlineStr">
+        <is>
+          <t>CAC 2026</t>
+        </is>
+      </c>
+      <c r="B33" s="45" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="46">
+        <f>F31/F33</f>
+        <v/>
+      </c>
+      <c r="E33" s="47" t="inlineStr">
+        <is>
+          <t>Inscrits 2026</t>
+        </is>
+      </c>
+      <c r="F33" s="48" t="n">
+        <v>1229</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>Lecture : les dépenses poussent le CAC de +34 € ; le volume supplémentaire l'amortit de −21 € ; net +13 €. La tension = l'effet dépenses &gt; l'effet volume.</t>
         </is>
       </c>
     </row>
@@ -2169,7 +2497,7 @@
       <c r="C6" s="19" t="n">
         <v>7525580</v>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="49">
         <f>C6/(B6+C6)</f>
         <v/>
       </c>
@@ -2186,7 +2514,7 @@
       <c r="C7" s="19" t="n">
         <v>4951430</v>
       </c>
-      <c r="D7" s="44">
+      <c r="D7" s="49">
         <f>C7/(B7+C7)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Bridge du CAC : axe tronqué + étiquettes -> les pas +34/-21 deviennent lisibles
Le waterfall partait de 0 : les bâtons pleins (341/353) écrasaient les pas
+34/-21. Correction : axe tronqué (320-385), gapWidth réduit, valeurs affichées
sur les barres. Les steps sont maintenant nets. (Option B = barres de
contribution autour de zéro, tenue en réserve.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/DEMO_ACTE1.xlsx
+++ b/eduservices/tagetik/DEMO_ACTE1.xlsx
@@ -824,6 +824,9 @@
               </a:ln>
             </spPr>
           </dPt>
+          <dLbls>
+            <showVal val="1"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Diagnostic CAC'!$A$30:$A$33</f>
@@ -835,7 +838,7 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="150"/>
+        <gapWidth val="45"/>
         <overlap val="100"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -855,9 +858,26 @@
         <axId val="100"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="385"/>
+          <min val="320"/>
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>CAC (€)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>

</xml_diff>

<commit_message>
Cockpit : remplacer le combo double-axe (trompeur) par base 100 dépenses vs inscrits
Le combo barres/courbe avait deux axes -> rapport visuel arbitraire (semblait
montrer inscrits > CAC). Remplacé par un graphe base 100 des dépenses vs inscrits
sur le MÊME axe : dépenses (ochre, +21%) décrochent au-dessus des inscrits (teal,
+12%), l'écart = la hausse du CAC. Honnête, pas de double-axe.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/DEMO_ACTE1.xlsx
+++ b/eduservices/tagetik/DEMO_ACTE1.xlsx
@@ -19,13 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.00,,&quot; M€&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="167" formatCode="&quot;▲ &quot;0.0%"/>
     <numFmt numFmtId="168" formatCode="&quot;▲ &quot;0.0&quot; pt&quot;"/>
     <numFmt numFmtId="169" formatCode="#,##0&quot; €&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="29">
     <font>
@@ -305,12 +306,12 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -430,16 +431,15 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Volume (inscrits, barres) vs coût par inscrit (CAC, courbe)</a:t>
+              <a:t>Dépenses (+21%) montent plus vite que les inscrits (+12%) — l'écart = la hausse du CAC</a:t>
             </a:r>
           </a:p>
         </rich>
       </tx>
     </title>
     <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
+      <lineChart>
+        <grouping val="standard"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -449,40 +449,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E4F0EC"/>
-            </a:solidFill>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$20:$D$20</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$21:$D$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'Cockpit'!A22</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="28000">
+            <a:ln w="30000">
               <a:solidFill>
                 <a:srgbClr val="B3641C"/>
               </a:solidFill>
@@ -497,6 +464,46 @@
               </a:ln>
             </spPr>
           </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$20:$D$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Cockpit'!$B$21:$D$21</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Cockpit'!A22</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="30000">
+              <a:solidFill>
+                <a:srgbClr val="0D7A62"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Cockpit'!$B$20:$D$20</f>
+            </numRef>
+          </cat>
           <val>
             <numRef>
               <f>'Cockpit'!$B$22:$D$22</f>
@@ -504,7 +511,7 @@
           </val>
         </ser>
         <axId val="10"/>
-        <axId val="200"/>
+        <axId val="100"/>
       </lineChart>
       <catAx>
         <axId val="10"/>
@@ -524,51 +531,9 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Inscrits</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-      </valAx>
-      <valAx>
-        <axId val="200"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>CAC (€)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
@@ -2026,63 +1991,68 @@
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
         <is>
-          <t>TENSION — le volume monte, mais le coût unitaire aussi</t>
+          <t>TENSION — base 100 en 2024</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="31" t="n">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Année</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="n">
         <v>2024</v>
       </c>
-      <c r="C20" s="31" t="n">
+      <c r="C20" s="32" t="n">
         <v>2025</v>
       </c>
-      <c r="D20" s="31" t="n">
+      <c r="D20" s="32" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Dépenses acq.</t>
+        </is>
+      </c>
+      <c r="B21" s="34">
+        <f>B15/$B15*100</f>
+        <v/>
+      </c>
+      <c r="C21" s="34">
+        <f>C15/$B15*100</f>
+        <v/>
+      </c>
+      <c r="D21" s="34">
+        <f>D15/$B15*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Inscrits</t>
         </is>
       </c>
-      <c r="B21" s="33">
-        <f>B14</f>
-        <v/>
-      </c>
-      <c r="C21" s="33">
-        <f>C14</f>
-        <v/>
-      </c>
-      <c r="D21" s="33">
-        <f>D14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="32" t="inlineStr">
-        <is>
-          <t>CAC (€)</t>
-        </is>
-      </c>
       <c r="B22" s="34">
-        <f>B16</f>
+        <f>B14/$B14*100</f>
         <v/>
       </c>
       <c r="C22" s="34">
-        <f>C16</f>
+        <f>C14/$B14*100</f>
         <v/>
       </c>
       <c r="D22" s="34">
-        <f>D16</f>
+        <f>D14/$B14*100</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>Les inscrits progressent (barres) mais le CAC grimpe (courbe) : les dépenses montent plus vite que le volume. Clic tuile CAC → Diagnostic.</t>
+          <t>Même base (100), même axe : les dépenses (ochre) décrochent au-dessus des inscrits (teal). L'écart = la dégradation du CAC. Clic tuile CAC → Diagnostic.</t>
         </is>
       </c>
     </row>

</xml_diff>